<commit_message>
feat(F-NAR-016): TREE-DIF-005 T1 moment du jour, T2 bac/échelle/herbe
Passe agent après premier apply. check OK. Désir: glisser.
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-005.xlsx
+++ b/stories/arbres/TREE-DIF-005.xlsx
@@ -1197,12 +1197,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Au bout du village, le parc s'ouvre. Un platane jette une ombre ronde. Des moineaux picorent près du bac. Le toboggan en métal brille un peu. Du sable fin colle déjà sur la rampe. Ça sent le soleil et la poussière. Tu vois le toboggan, Aniss ? Oui, papa. Il brille. Le banc est encore un peu froid. En ce moment, Aniss tire sa chaussure. Je veux glisser ! Nino est déjà près de l'échelle. Ses lèvres bougent, tout lentement. Je veux le. On l'écoute, Aniss ? Oui.</t>
+          <t>Au bout du village, le parc s'ouvre. Un platane jette une ombre ronde. Des moineaux picorent près du bac. Le toboggan en métal brille un peu. Du sable fin colle déjà sur la rampe. Ça sent le soleil et la poussière. Tu vois le toboggan, Aniss ? Oui, papa. Il brille. Le banc est encore un peu froid. En ce moment, Aniss tire sa chaussure. Je veux glisser ! Nino est déjà près de l'échelle. Ses lèvres bougent, tout lentement. Je veux le. Nino te parle, Aniss ? Oui.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Au bout du village, le parc s'ouvre. Un platane jette une ombre ronde. Des moineaux picorent près du bac. Le toboggan en métal brille un peu. Du sable fin colle déjà sur la rampe. Ça sent le soleil et la poussière. Tu vois le toboggan, Aniss ? Oui, papa. Il brille. Le banc est encore un peu froid. En ce moment, Aniss tire sa chaussure. Je veux glisser ! Nino est déjà près de l'échelle. Ses lèvres bougent, tout lentement. Je veux le. On l'écoute, Aniss ? Oui.</t>
+          <t>Au bout du village, le parc s'ouvre. Un platane jette une ombre ronde. Des moineaux picorent près du bac. Le toboggan en métal brille un peu. Du sable fin colle déjà sur la rampe. Ça sent le soleil et la poussière. Tu vois le toboggan, Aniss ? Oui, papa. Il brille. Le banc est encore un peu froid. En ce moment, Aniss tire sa chaussure. Je veux glisser ! Nino est déjà près de l'échelle. Ses lèvres bougent, tout lentement. Je veux le. Nino te parle, Aniss ? Oui.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1348,7 +1348,7 @@
 narrateur|Nino est déjà près de l'échelle.
 narrateur|Ses lèvres bougent, tout lentement.
 copain|Je veux le.
-papa|On l'écoute, Aniss ?
+papa|Nino te parle, Aniss ?
 enfant-m|Oui.</t>
         </is>
       </c>
@@ -1938,12 +1938,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Nino reprend, tout doux. Le toboggan a du sable. J'ai attendu. Merci, Aniss. On peut avancer, maintenant. L'ombre du platane est longue. Où va-t-on d'abord ?</t>
+          <t>Nino reprend, tout doux. Le toboggan a du sable. On y va. Merci, Aniss. On peut avancer, maintenant. L'ombre du platane est longue. Où va-t-on d'abord ?</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Nino reprend, tout doux. Le toboggan a du sable. J'ai attendu. Merci, Aniss. On peut avancer, maintenant. L'ombre du platane est longue. Où va-t-on d'abord ?</t>
+          <t>Nino reprend, tout doux. Le toboggan a du sable. On y va. Merci, Aniss. On peut avancer, maintenant. L'ombre du platane est longue. Où va-t-on d'abord ?</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -2080,7 +2080,7 @@
         <is>
           <t>narrateur|Nino reprend, tout doux.
 copain|Le toboggan a du sable.
-enfant-m|J'ai attendu.
+enfant-m|On y va.
 papa|Merci, Aniss.
 maman|On peut avancer, maintenant.
 narrateur|L'ombre du platane est longue.
@@ -2680,12 +2680,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Du sable froid remplit le bac. Un rond rouge dépasse, à peine. Le ballon est. Aniss creuse, tout doux, et attend. Il est sous le sable ? Le ballon est sous le sable. Je le sors. Le rouge sort, un peu sablé. Les doigts d'Aniss sont un peu rouges. Vous l'avez, tous les deux. Maintenant, le toboggan ! Ils portent le ballon vers l'échelle.</t>
+          <t>Du sable froid remplit le bac. Un rond rouge dépasse, à peine. Le ballon est. Aniss creuse, tout doux, et attend. Il est sous le sable ? Le ballon est sous le sable. Je le sors. Le rouge sort, un peu sablé. Les doigts d'Aniss sont un peu rouges. Vous l'avez, tous les deux. Ils grimpent, le ballon contre la hanche. Puis ça file, tout court, tout vif.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Du sable froid remplit le bac. Un rond rouge dépasse, à peine. Le ballon est. Aniss creuse, tout doux, et attend. Il est sous le sable ? Le ballon est sous le sable. Je le sors. Le rouge sort, un peu sablé. Les doigts d'Aniss sont un peu rouges. Vous l'avez, tous les deux. Maintenant, le toboggan ! Ils portent le ballon vers l'échelle.</t>
+          <t>Du sable froid remplit le bac. Un rond rouge dépasse, à peine. Le ballon est. Aniss creuse, tout doux, et attend. Il est sous le sable ? Le ballon est sous le sable. Je le sors. Le rouge sort, un peu sablé. Les doigts d'Aniss sont un peu rouges. Vous l'avez, tous les deux. Ils grimpent, le ballon contre la hanche. Puis ça file, tout court, tout vif.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -2826,8 +2826,8 @@
 narrateur|Le rouge sort, un peu sablé.
 narrateur|Les doigts d'Aniss sont un peu rouges.
 maman|Vous l'avez, tous les deux.
-enfant-m|Maintenant, le toboggan !
-narrateur|Ils portent le ballon vers l'échelle.</t>
+narrateur|Ils grimpent, le ballon contre la hanche.
+narrateur|Puis ça file, tout court, tout vif.</t>
         </is>
       </c>
       <c r="AX10" t="inlineStr">
@@ -3039,12 +3039,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>La rosée brille encore sur l'herbe. Le seau bleu attend près du bac. Le seau est. Aniss tient l'anse, sans tirer. Il va le dire. Le seau est lourd. On verse, alors. Ils raclent le sable de la rampe. Le bleu se remplit, grain après grain. Sous les doigts, le métal pique un peu. La rampe redevient lisse. On peut glisser !</t>
+          <t>La rosée brille encore sur l'herbe. Le seau bleu attend près du bac. Le seau est. Aniss tient l'anse, sans tirer. Il va le dire. Le seau est lourd. On verse, alors. Ils raclent le sable de la rampe. Le bleu se remplit, grain après grain. Sous les doigts, le métal pique un peu. La rampe redevient lisse. Ça file, tout d'un coup.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>La rosée brille encore sur l'herbe. Le seau bleu attend près du bac. Le seau est. Aniss tient l'anse, sans tirer. Il va le dire. Le seau est lourd. On verse, alors. Ils raclent le sable de la rampe. Le bleu se remplit, grain après grain. Sous les doigts, le métal pique un peu. La rampe redevient lisse. On peut glisser !</t>
+          <t>La rosée brille encore sur l'herbe. Le seau bleu attend près du bac. Le seau est. Aniss tient l'anse, sans tirer. Il va le dire. Le seau est lourd. On verse, alors. Ils raclent le sable de la rampe. Le bleu se remplit, grain après grain. Sous les doigts, le métal pique un peu. La rampe redevient lisse. Ça file, tout d'un coup.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -3186,7 +3186,7 @@
 narrateur|Le bleu se remplit, grain après grain.
 narrateur|Sous les doigts, le métal pique un peu.
 papa|La rampe redevient lisse.
-enfant-m|On peut glisser !</t>
+narrateur|Ça file, tout d'un coup.</t>
         </is>
       </c>
       <c r="AX12" t="inlineStr">
@@ -3398,12 +3398,12 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>L'ombre du platane est longue. Le doudou dort dans le bac, tout sablé. Le doudou est. Aniss garde les mains, et attend. Il le veut, ce doudou ? Le doudou est tout sablé. On le tapote. Le sable tombe, un nuage minuscule. Nino le serre contre sa joue. Un moineau crie, tout près. Il est prêt, maintenant. On grimpe, avec lui.</t>
+          <t>L'ombre du platane est longue. Le doudou dort dans le bac, tout sablé. Le doudou est. Aniss garde les mains, et attend. Il le veut, ce doudou ? Le doudou est tout sablé. On le tapote. Le sable tombe, un nuage minuscule. Nino le serre contre sa joue. Un moineau crie, tout près. Il est prêt, maintenant. Ils glissent, le doudou entre eux.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>L'ombre du platane est longue. Le doudou dort dans le bac, tout sablé. Le doudou est. Aniss garde les mains, et attend. Il le veut, ce doudou ? Le doudou est tout sablé. On le tapote. Le sable tombe, un nuage minuscule. Nino le serre contre sa joue. Un moineau crie, tout près. Il est prêt, maintenant. On grimpe, avec lui.</t>
+          <t>L'ombre du platane est longue. Le doudou dort dans le bac, tout sablé. Le doudou est. Aniss garde les mains, et attend. Il le veut, ce doudou ? Le doudou est tout sablé. On le tapote. Le sable tombe, un nuage minuscule. Nino le serre contre sa joue. Un moineau crie, tout près. Il est prêt, maintenant. Ils glissent, le doudou entre eux.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -3545,7 +3545,7 @@
 narrateur|Nino le serre contre sa joue.
 narrateur|Un moineau crie, tout près.
 maman|Il est prêt, maintenant.
-enfant-m|On grimpe, avec lui.</t>
+narrateur|Ils glissent, le doudou entre eux.</t>
         </is>
       </c>
       <c r="AX14" t="inlineStr">
@@ -4128,12 +4128,12 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Sous les doigts, le métal pique un peu. Le ballon rouge coince un barreau. Le ballon va. Aniss ouvre les mains, en bas, et attend. Tu le laisses dire ? Le ballon va tomber. Je suis là. Nino pousse, tout doux. Le rouge atterrit dans les mains d'Aniss. Un moineau crie, tout près. Le chemin est libre. On monte, puis on glisse !</t>
+          <t>Sous les doigts, le métal pique un peu. Le ballon rouge coince un barreau. Le ballon va. Aniss ouvre les mains, en bas, et attend. Tu le laisses dire ? Le ballon va tomber. Je suis là. Nino pousse, tout doux. Le rouge atterrit dans les mains d'Aniss. Un moineau crie, tout près. Le chemin est libre. Ils montent, puis ça dévale.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Sous les doigts, le métal pique un peu. Le ballon rouge coince un barreau. Le ballon va. Aniss ouvre les mains, en bas, et attend. Tu le laisses dire ? Le ballon va tomber. Je suis là. Nino pousse, tout doux. Le rouge atterrit dans les mains d'Aniss. Un moineau crie, tout près. Le chemin est libre. On monte, puis on glisse !</t>
+          <t>Sous les doigts, le métal pique un peu. Le ballon rouge coince un barreau. Le ballon va. Aniss ouvre les mains, en bas, et attend. Tu le laisses dire ? Le ballon va tomber. Je suis là. Nino pousse, tout doux. Le rouge atterrit dans les mains d'Aniss. Un moineau crie, tout près. Le chemin est libre. Ils montent, puis ça dévale.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -4275,7 +4275,7 @@
 narrateur|Le rouge atterrit dans les mains d'Aniss.
 narrateur|Un moineau crie, tout près.
 papa|Le chemin est libre.
-enfant-m|On monte, puis on glisse !</t>
+narrateur|Ils montent, puis ça dévale.</t>
         </is>
       </c>
       <c r="AX18" t="inlineStr">
@@ -4487,12 +4487,12 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>L'ombre du platane est longue. Le seau bleu pend près du haut. Le seau va. Aniss reste un barreau plus bas. On l'écoute, d'accord ? Le seau va nous aider. Je te le tends. Nino pousse le sable, tout lentement. Les grains tombent dans le bleu. Du sable froid remplit le bac. La rampe redevient glissante. À nous !</t>
+          <t>L'ombre du platane est longue. Le seau bleu pend près du haut. Le seau va. Aniss reste un barreau plus bas. On l'écoute, d'accord ? Le seau va nous aider. Je te le tends. Nino pousse le sable, tout lentement. Les grains tombent dans le bleu. Du sable froid remplit le bac. La rampe redevient glissante. Ils dévalent, le seau à la main.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>L'ombre du platane est longue. Le seau bleu pend près du haut. Le seau va. Aniss reste un barreau plus bas. On l'écoute, d'accord ? Le seau va nous aider. Je te le tends. Nino pousse le sable, tout lentement. Les grains tombent dans le bleu. Du sable froid remplit le bac. La rampe redevient glissante. À nous !</t>
+          <t>L'ombre du platane est longue. Le seau bleu pend près du haut. Le seau va. Aniss reste un barreau plus bas. On l'écoute, d'accord ? Le seau va nous aider. Je te le tends. Nino pousse le sable, tout lentement. Les grains tombent dans le bleu. Du sable froid remplit le bac. La rampe redevient glissante. Ils dévalent, le seau à la main.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -4634,7 +4634,7 @@
 narrateur|Les grains tombent dans le bleu.
 narrateur|Du sable froid remplit le bac.
 maman|La rampe redevient glissante.
-enfant-m|À nous !</t>
+narrateur|Ils dévalent, le seau à la main.</t>
         </is>
       </c>
       <c r="AX20" t="inlineStr">
@@ -4846,12 +4846,12 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>La rosée brille encore sur l'herbe. Le doudou est coincé sur un barreau. Le doudou va. Aniss ne le prend pas, et attend. Sa phrase n'est pas finie. Le doudou va avec moi. Je te le passe. Nino le glisse sous son bras. Ils montent, barreau après barreau. Sous les doigts, le métal pique un peu. Vous y êtes, tout en haut. On glisse ensemble !</t>
+          <t>La rosée brille encore sur l'herbe. Le doudou est coincé sur un barreau. Le doudou va. Aniss ne le prend pas, et attend. Il cherche encore. Le doudou va avec moi. Je te le passe. Nino le glisse sous son bras. Ils montent, barreau après barreau. Sous les doigts, le métal pique un peu. Vous y êtes, tout en haut. Ils glissent, le doudou au milieu.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>La rosée brille encore sur l'herbe. Le doudou est coincé sur un barreau. Le doudou va. Aniss ne le prend pas, et attend. Sa phrase n'est pas finie. Le doudou va avec moi. Je te le passe. Nino le glisse sous son bras. Ils montent, barreau après barreau. Sous les doigts, le métal pique un peu. Vous y êtes, tout en haut. On glisse ensemble !</t>
+          <t>La rosée brille encore sur l'herbe. Le doudou est coincé sur un barreau. Le doudou va. Aniss ne le prend pas, et attend. Il cherche encore. Le doudou va avec moi. Je te le passe. Nino le glisse sous son bras. Ils montent, barreau après barreau. Sous les doigts, le métal pique un peu. Vous y êtes, tout en haut. Ils glissent, le doudou au milieu.</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -4986,14 +4986,14 @@
 narrateur|Le doudou est coincé sur un barreau.
 copain|Le doudou va.
 narrateur|Aniss ne le prend pas, et attend.
-maman|Sa phrase n'est pas finie.
+maman|Il cherche encore.
 copain|Le doudou va avec moi.
 enfant-m|Je te le passe.
 narrateur|Nino le glisse sous son bras.
 narrateur|Ils montent, barreau après barreau.
 narrateur|Sous les doigts, le métal pique un peu.
 papa|Vous y êtes, tout en haut.
-enfant-m|On glisse ensemble !</t>
+narrateur|Ils glissent, le doudou au milieu.</t>
         </is>
       </c>
       <c r="AX22" t="inlineStr">
@@ -6653,12 +6653,12 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>La lumière pèse, toute blanche. Au toucher, le toboggan est tiède. Sous les paumes, le sable brûle un peu. Je veux glisser, vite ! Nino parle, tout bas, tout lent. Le bac est. Aniss se tait, les mains au barreau. Tu l'entends, ce murmure ? Oui, maman. C'est Nino. Le parc dore, après la sieste. Une cigale frotte, tout loin. J'attends sa phrase.</t>
+          <t>La lumière pèse, toute blanche. Au toucher, le toboggan est tiède. Sous les paumes, le sable brûle un peu. Je veux glisser, vite ! Nino parle, tout bas, tout lent. Le bac est. Aniss se tait, les mains au barreau. Tu l'entends, ce murmure ? Oui, maman. C'est Nino. Le parc dore, après la sieste. Une cigale frotte, tout loin. J'attends.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>La lumière pèse, toute blanche. Au toucher, le toboggan est tiède. Sous les paumes, le sable brûle un peu. Je veux glisser, vite ! Nino parle, tout bas, tout lent. Le bac est. Aniss se tait, les mains au barreau. Tu l'entends, ce murmure ? Oui, maman. C'est Nino. Le parc dore, après la sieste. Une cigale frotte, tout loin. J'attends sa phrase.</t>
+          <t>La lumière pèse, toute blanche. Au toucher, le toboggan est tiède. Sous les paumes, le sable brûle un peu. Je veux glisser, vite ! Nino parle, tout bas, tout lent. Le bac est. Aniss se tait, les mains au barreau. Tu l'entends, ce murmure ? Oui, maman. C'est Nino. Le parc dore, après la sieste. Une cigale frotte, tout loin. J'attends.</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -6805,7 +6805,7 @@
 enfant-m|C'est Nino.
 papa|Le parc dore, après la sieste.
 narrateur|Une cigale frotte, tout loin.
-enfant-m|J'attends sa phrase.</t>
+enfant-m|J'attends.</t>
         </is>
       </c>
       <c r="AX32" t="inlineStr">
@@ -7020,12 +7020,12 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Nino reprend, tout doux. Le bac est plein. J'ai attendu. Merci, Aniss. On peut avancer, maintenant. La lumière pèse, toute blanche. Où va-t-on d'abord ?</t>
+          <t>Nino reprend, tout doux. Le bac est plein. On y va. Merci, Aniss. On peut avancer, maintenant. La lumière pèse, toute blanche. Où va-t-on d'abord ?</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Nino reprend, tout doux. Le bac est plein. J'ai attendu. Merci, Aniss. On peut avancer, maintenant. La lumière pèse, toute blanche. Où va-t-on d'abord ?</t>
+          <t>Nino reprend, tout doux. Le bac est plein. On y va. Merci, Aniss. On peut avancer, maintenant. La lumière pèse, toute blanche. Où va-t-on d'abord ?</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -7162,7 +7162,7 @@
         <is>
           <t>narrateur|Nino reprend, tout doux.
 copain|Le bac est plein.
-enfant-m|J'ai attendu.
+enfant-m|On y va.
 papa|Merci, Aniss.
 maman|On peut avancer, maintenant.
 narrateur|La lumière pèse, toute blanche.
@@ -7762,12 +7762,12 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Sous les paumes, le sable brûle un peu. Un rond rouge dépasse, à peine. Le ballon est. Aniss creuse, tout doux, et attend. Il est sous le sable ? Le ballon est sous le sable. Je le sors. Le rouge sort, un peu sablé. Une goutte coule sur la tempe d'Aniss. Vous l'avez, tous les deux. Maintenant, le toboggan ! Ils portent le ballon vers l'échelle.</t>
+          <t>Sous les paumes, le sable brûle un peu. Un rond rouge dépasse, à peine. Le ballon est. Aniss creuse, tout doux, et attend. Il est sous le sable ? Le ballon est sous le sable. Je le sors. Le rouge sort, un peu sablé. Une goutte coule sur la tempe d'Aniss. Vous l'avez, tous les deux. Ils grimpent, le ballon contre la hanche. Puis ça file, tout court, tout vif.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Sous les paumes, le sable brûle un peu. Un rond rouge dépasse, à peine. Le ballon est. Aniss creuse, tout doux, et attend. Il est sous le sable ? Le ballon est sous le sable. Je le sors. Le rouge sort, un peu sablé. Une goutte coule sur la tempe d'Aniss. Vous l'avez, tous les deux. Maintenant, le toboggan ! Ils portent le ballon vers l'échelle.</t>
+          <t>Sous les paumes, le sable brûle un peu. Un rond rouge dépasse, à peine. Le ballon est. Aniss creuse, tout doux, et attend. Il est sous le sable ? Le ballon est sous le sable. Je le sors. Le rouge sort, un peu sablé. Une goutte coule sur la tempe d'Aniss. Vous l'avez, tous les deux. Ils grimpent, le ballon contre la hanche. Puis ça file, tout court, tout vif.</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -7908,8 +7908,8 @@
 narrateur|Le rouge sort, un peu sablé.
 narrateur|Une goutte coule sur la tempe d'Aniss.
 maman|Vous l'avez, tous les deux.
-enfant-m|Maintenant, le toboggan !
-narrateur|Ils portent le ballon vers l'échelle.</t>
+narrateur|Ils grimpent, le ballon contre la hanche.
+narrateur|Puis ça file, tout court, tout vif.</t>
         </is>
       </c>
       <c r="AX38" t="inlineStr">
@@ -8121,12 +8121,12 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>L'air sent la poussière chaude. Le seau bleu attend près du bac. Le seau est. Aniss tient l'anse, sans tirer. Il va le dire. Le seau est lourd. On verse, alors. Ils raclent le sable de la rampe. Le bleu se remplit, grain après grain. Au toucher, le toboggan est tiède. La rampe redevient lisse. On peut glisser !</t>
+          <t>L'air sent la poussière chaude. Le seau bleu attend près du bac. Le seau est. Aniss tient l'anse, sans tirer. Il va le dire. Le seau est lourd. On verse, alors. Ils raclent le sable de la rampe. Le bleu se remplit, grain après grain. Au toucher, le toboggan est tiède. La rampe redevient lisse. Ça file, tout d'un coup.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>L'air sent la poussière chaude. Le seau bleu attend près du bac. Le seau est. Aniss tient l'anse, sans tirer. Il va le dire. Le seau est lourd. On verse, alors. Ils raclent le sable de la rampe. Le bleu se remplit, grain après grain. Au toucher, le toboggan est tiède. La rampe redevient lisse. On peut glisser !</t>
+          <t>L'air sent la poussière chaude. Le seau bleu attend près du bac. Le seau est. Aniss tient l'anse, sans tirer. Il va le dire. Le seau est lourd. On verse, alors. Ils raclent le sable de la rampe. Le bleu se remplit, grain après grain. Au toucher, le toboggan est tiède. La rampe redevient lisse. Ça file, tout d'un coup.</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -8268,7 +8268,7 @@
 narrateur|Le bleu se remplit, grain après grain.
 narrateur|Au toucher, le toboggan est tiède.
 papa|La rampe redevient lisse.
-enfant-m|On peut glisser !</t>
+narrateur|Ça file, tout d'un coup.</t>
         </is>
       </c>
       <c r="AX40" t="inlineStr">
@@ -8480,12 +8480,12 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>La lumière pèse, toute blanche. Le doudou dort dans le bac, tout sablé. Le doudou est. Aniss garde les mains, et attend. Il le veut, ce doudou ? Le doudou est tout sablé. On le tapote. Le sable tombe, un nuage minuscule. Nino le serre contre sa joue. Une cigale frotte, tout loin. Il est prêt, maintenant. On grimpe, avec lui.</t>
+          <t>La lumière pèse, toute blanche. Le doudou dort dans le bac, tout sablé. Le doudou est. Aniss garde les mains, et attend. Il le veut, ce doudou ? Le doudou est tout sablé. On le tapote. Le sable tombe, un nuage minuscule. Nino le serre contre sa joue. Une cigale frotte, tout loin. Il est prêt, maintenant. Ils glissent, le doudou entre eux.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>La lumière pèse, toute blanche. Le doudou dort dans le bac, tout sablé. Le doudou est. Aniss garde les mains, et attend. Il le veut, ce doudou ? Le doudou est tout sablé. On le tapote. Le sable tombe, un nuage minuscule. Nino le serre contre sa joue. Une cigale frotte, tout loin. Il est prêt, maintenant. On grimpe, avec lui.</t>
+          <t>La lumière pèse, toute blanche. Le doudou dort dans le bac, tout sablé. Le doudou est. Aniss garde les mains, et attend. Il le veut, ce doudou ? Le doudou est tout sablé. On le tapote. Le sable tombe, un nuage minuscule. Nino le serre contre sa joue. Une cigale frotte, tout loin. Il est prêt, maintenant. Ils glissent, le doudou entre eux.</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -8627,7 +8627,7 @@
 narrateur|Nino le serre contre sa joue.
 narrateur|Une cigale frotte, tout loin.
 maman|Il est prêt, maintenant.
-enfant-m|On grimpe, avec lui.</t>
+narrateur|Ils glissent, le doudou entre eux.</t>
         </is>
       </c>
       <c r="AX42" t="inlineStr">
@@ -9210,12 +9210,12 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Au toucher, le toboggan est tiède. Le ballon rouge coince un barreau. Le ballon va. Aniss ouvre les mains, en bas, et attend. Tu le laisses dire ? Le ballon va tomber. Je suis là. Nino pousse, tout doux. Le rouge atterrit dans les mains d'Aniss. Une cigale frotte, tout loin. Le chemin est libre. On monte, puis on glisse !</t>
+          <t>Au toucher, le toboggan est tiède. Le ballon rouge coince un barreau. Le ballon va. Aniss ouvre les mains, en bas, et attend. Tu le laisses dire ? Le ballon va tomber. Je suis là. Nino pousse, tout doux. Le rouge atterrit dans les mains d'Aniss. Une cigale frotte, tout loin. Le chemin est libre. Ils montent, puis ça dévale.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Au toucher, le toboggan est tiède. Le ballon rouge coince un barreau. Le ballon va. Aniss ouvre les mains, en bas, et attend. Tu le laisses dire ? Le ballon va tomber. Je suis là. Nino pousse, tout doux. Le rouge atterrit dans les mains d'Aniss. Une cigale frotte, tout loin. Le chemin est libre. On monte, puis on glisse !</t>
+          <t>Au toucher, le toboggan est tiède. Le ballon rouge coince un barreau. Le ballon va. Aniss ouvre les mains, en bas, et attend. Tu le laisses dire ? Le ballon va tomber. Je suis là. Nino pousse, tout doux. Le rouge atterrit dans les mains d'Aniss. Une cigale frotte, tout loin. Le chemin est libre. Ils montent, puis ça dévale.</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -9357,7 +9357,7 @@
 narrateur|Le rouge atterrit dans les mains d'Aniss.
 narrateur|Une cigale frotte, tout loin.
 papa|Le chemin est libre.
-enfant-m|On monte, puis on glisse !</t>
+narrateur|Ils montent, puis ça dévale.</t>
         </is>
       </c>
       <c r="AX46" t="inlineStr">
@@ -9569,12 +9569,12 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>La lumière pèse, toute blanche. Le seau bleu pend près du haut. Le seau va. Aniss reste un barreau plus bas. On l'écoute, d'accord ? Le seau va nous aider. Je te le tends. Nino pousse le sable, tout lentement. Les grains tombent dans le bleu. Sous les paumes, le sable brûle un peu. La rampe redevient glissante. À nous !</t>
+          <t>La lumière pèse, toute blanche. Le seau bleu pend près du haut. Le seau va. Aniss reste un barreau plus bas. On l'écoute, d'accord ? Le seau va nous aider. Je te le tends. Nino pousse le sable, tout lentement. Les grains tombent dans le bleu. Sous les paumes, le sable brûle un peu. La rampe redevient glissante. Ils dévalent, le seau à la main.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>La lumière pèse, toute blanche. Le seau bleu pend près du haut. Le seau va. Aniss reste un barreau plus bas. On l'écoute, d'accord ? Le seau va nous aider. Je te le tends. Nino pousse le sable, tout lentement. Les grains tombent dans le bleu. Sous les paumes, le sable brûle un peu. La rampe redevient glissante. À nous !</t>
+          <t>La lumière pèse, toute blanche. Le seau bleu pend près du haut. Le seau va. Aniss reste un barreau plus bas. On l'écoute, d'accord ? Le seau va nous aider. Je te le tends. Nino pousse le sable, tout lentement. Les grains tombent dans le bleu. Sous les paumes, le sable brûle un peu. La rampe redevient glissante. Ils dévalent, le seau à la main.</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -9716,7 +9716,7 @@
 narrateur|Les grains tombent dans le bleu.
 narrateur|Sous les paumes, le sable brûle un peu.
 maman|La rampe redevient glissante.
-enfant-m|À nous !</t>
+narrateur|Ils dévalent, le seau à la main.</t>
         </is>
       </c>
       <c r="AX48" t="inlineStr">
@@ -9928,12 +9928,12 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>L'air sent la poussière chaude. Le doudou est coincé sur un barreau. Le doudou va. Aniss ne le prend pas, et attend. Sa phrase n'est pas finie. Le doudou va avec moi. Je te le passe. Nino le glisse sous son bras. Ils montent, barreau après barreau. Au toucher, le toboggan est tiède. Vous y êtes, tout en haut. On glisse ensemble !</t>
+          <t>L'air sent la poussière chaude. Le doudou est coincé sur un barreau. Le doudou va. Aniss ne le prend pas, et attend. Il cherche encore. Le doudou va avec moi. Je te le passe. Nino le glisse sous son bras. Ils montent, barreau après barreau. Au toucher, le toboggan est tiède. Vous y êtes, tout en haut. Ils glissent, le doudou au milieu.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>L'air sent la poussière chaude. Le doudou est coincé sur un barreau. Le doudou va. Aniss ne le prend pas, et attend. Sa phrase n'est pas finie. Le doudou va avec moi. Je te le passe. Nino le glisse sous son bras. Ils montent, barreau après barreau. Au toucher, le toboggan est tiède. Vous y êtes, tout en haut. On glisse ensemble !</t>
+          <t>L'air sent la poussière chaude. Le doudou est coincé sur un barreau. Le doudou va. Aniss ne le prend pas, et attend. Il cherche encore. Le doudou va avec moi. Je te le passe. Nino le glisse sous son bras. Ils montent, barreau après barreau. Au toucher, le toboggan est tiède. Vous y êtes, tout en haut. Ils glissent, le doudou au milieu.</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -10068,14 +10068,14 @@
 narrateur|Le doudou est coincé sur un barreau.
 copain|Le doudou va.
 narrateur|Aniss ne le prend pas, et attend.
-maman|Sa phrase n'est pas finie.
+maman|Il cherche encore.
 copain|Le doudou va avec moi.
 enfant-m|Je te le passe.
 narrateur|Nino le glisse sous son bras.
 narrateur|Ils montent, barreau après barreau.
 narrateur|Au toucher, le toboggan est tiède.
 papa|Vous y êtes, tout en haut.
-enfant-m|On glisse ensemble !</t>
+narrateur|Ils glissent, le doudou au milieu.</t>
         </is>
       </c>
       <c r="AX50" t="inlineStr">
@@ -11739,12 +11739,12 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>La lumière devient orange, tout doux. Un lampadaire fait un petit tic. Le sable colle sur le toboggan. Je veux glisser avant la nuit ! Nino cherche encore un mot. Je rentre avec. Aniss attend, tout calme. Le métal refroidit, ce soir. Tu vois le sable, Aniss ? Oui. Sur le toboggan. L'ombre violette touche déjà l'herbe. On glisse après sa phrase.</t>
+          <t>La lumière devient orange, tout doux. Un lampadaire fait un petit tic. Le sable colle sur le toboggan. Je veux glisser avant la nuit ! Nino cherche encore un mot. Je glisse avec. Aniss attend, tout calme. Le métal refroidit, ce soir. Tu vois le sable, Aniss ? Oui. Sur le toboggan. L'ombre violette touche déjà l'herbe. On glisse après.</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>La lumière devient orange, tout doux. Un lampadaire fait un petit tic. Le sable colle sur le toboggan. Je veux glisser avant la nuit ! Nino cherche encore un mot. Je rentre avec. Aniss attend, tout calme. Le métal refroidit, ce soir. Tu vois le sable, Aniss ? Oui. Sur le toboggan. L'ombre violette touche déjà l'herbe. On glisse après sa phrase.</t>
+          <t>La lumière devient orange, tout doux. Un lampadaire fait un petit tic. Le sable colle sur le toboggan. Je veux glisser avant la nuit ! Nino cherche encore un mot. Je glisse avec. Aniss attend, tout calme. Le métal refroidit, ce soir. Tu vois le sable, Aniss ? Oui. Sur le toboggan. L'ombre violette touche déjà l'herbe. On glisse après.</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -11880,14 +11880,14 @@
 narrateur|Le sable colle sur le toboggan.
 enfant-m|Je veux glisser avant la nuit !
 narrateur|Nino cherche encore un mot.
-copain|Je rentre avec.
+copain|Je glisse avec.
 narrateur|Aniss attend, tout calme.
 papa|Le métal refroidit, ce soir.
 maman|Tu vois le sable, Aniss ?
 enfant-m|Oui.
 enfant-m|Sur le toboggan.
 narrateur|L'ombre violette touche déjà l'herbe.
-enfant-m|On glisse après sa phrase.</t>
+enfant-m|On glisse après.</t>
         </is>
       </c>
       <c r="AX60" t="inlineStr">
@@ -12102,12 +12102,12 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Nino reprend, tout doux. Je rentre avec toi. J'ai attendu. Merci, Aniss. On peut avancer, maintenant. L'ombre violette touche déjà l'herbe. Où va-t-on d'abord ?</t>
+          <t>Nino reprend, tout doux. Je glisse avec toi. On y va. Merci, Aniss. On peut avancer, maintenant. L'ombre violette touche déjà l'herbe. Où va-t-on d'abord ?</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Nino reprend, tout doux. Je rentre avec toi. J'ai attendu. Merci, Aniss. On peut avancer, maintenant. L'ombre violette touche déjà l'herbe. Où va-t-on d'abord ?</t>
+          <t>Nino reprend, tout doux. Je glisse avec toi. On y va. Merci, Aniss. On peut avancer, maintenant. L'ombre violette touche déjà l'herbe. Où va-t-on d'abord ?</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -12243,8 +12243,8 @@
       <c r="AW62" t="inlineStr">
         <is>
           <t>narrateur|Nino reprend, tout doux.
-copain|Je rentre avec toi.
-enfant-m|J'ai attendu.
+copain|Je glisse avec toi.
+enfant-m|On y va.
 papa|Merci, Aniss.
 maman|On peut avancer, maintenant.
 narrateur|L'ombre violette touche déjà l'herbe.
@@ -12844,12 +12844,12 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Voilà le sable, déjà refroidi, tout fin. Un rond rouge dépasse, à peine. Le ballon est. Aniss creuse, tout doux, et attend. Il est sous le sable ? Le ballon est sous le sable. Je le sors. Le rouge sort, un peu sablé. Les genoux d'Aniss ont du sable froid. Vous l'avez, tous les deux. Maintenant, le toboggan ! Ils portent le ballon vers l'échelle.</t>
+          <t>Voilà le sable, déjà refroidi, tout fin. Un rond rouge dépasse, à peine. Le ballon est. Aniss creuse, tout doux, et attend. Il est sous le sable ? Le ballon est sous le sable. Je le sors. Le rouge sort, un peu sablé. Les genoux d'Aniss ont du sable froid. Vous l'avez, tous les deux. Ils grimpent, le ballon contre la hanche. Puis ça file, tout court, tout vif.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Voilà le sable, déjà refroidi, tout fin. Un rond rouge dépasse, à peine. Le ballon est. Aniss creuse, tout doux, et attend. Il est sous le sable ? Le ballon est sous le sable. Je le sors. Le rouge sort, un peu sablé. Les genoux d'Aniss ont du sable froid. Vous l'avez, tous les deux. Maintenant, le toboggan ! Ils portent le ballon vers l'échelle.</t>
+          <t>Voilà le sable, déjà refroidi, tout fin. Un rond rouge dépasse, à peine. Le ballon est. Aniss creuse, tout doux, et attend. Il est sous le sable ? Le ballon est sous le sable. Je le sors. Le rouge sort, un peu sablé. Les genoux d'Aniss ont du sable froid. Vous l'avez, tous les deux. Ils grimpent, le ballon contre la hanche. Puis ça file, tout court, tout vif.</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -12994,8 +12994,8 @@
 narrateur|Le rouge sort, un peu sablé.
 narrateur|Les genoux d'Aniss ont du sable froid.
 maman|Vous l'avez, tous les deux.
-enfant-m|Maintenant, le toboggan !
-narrateur|Ils portent le ballon vers l'échelle.</t>
+narrateur|Ils grimpent, le ballon contre la hanche.
+narrateur|Puis ça file, tout court, tout vif.</t>
         </is>
       </c>
       <c r="AX66" t="inlineStr">
@@ -13207,12 +13207,12 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>La lumière devient orange, tout doux. Le seau bleu attend près du bac. Le seau est. Aniss tient l'anse, sans tirer. Il va le dire. Le seau est lourd. On verse, alors. Ils raclent le sable de la rampe. Le bleu se remplit, grain après grain. Maintenant le toboggan refroidit. La rampe redevient lisse. On peut glisser !</t>
+          <t>La lumière devient orange, tout doux. Le seau bleu attend près du bac. Le seau est. Aniss tient l'anse, sans tirer. Il va le dire. Le seau est lourd. On verse, alors. Ils raclent le sable de la rampe. Le bleu se remplit, grain après grain. Maintenant le toboggan refroidit. La rampe redevient lisse. Ça file, tout d'un coup.</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>La lumière devient orange, tout doux. Le seau bleu attend près du bac. Le seau est. Aniss tient l'anse, sans tirer. Il va le dire. Le seau est lourd. On verse, alors. Ils raclent le sable de la rampe. Le bleu se remplit, grain après grain. Maintenant le toboggan refroidit. La rampe redevient lisse. On peut glisser !</t>
+          <t>La lumière devient orange, tout doux. Le seau bleu attend près du bac. Le seau est. Aniss tient l'anse, sans tirer. Il va le dire. Le seau est lourd. On verse, alors. Ils raclent le sable de la rampe. Le bleu se remplit, grain après grain. Maintenant le toboggan refroidit. La rampe redevient lisse. Ça file, tout d'un coup.</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -13354,7 +13354,7 @@
 narrateur|Le bleu se remplit, grain après grain.
 narrateur|Maintenant le toboggan refroidit.
 papa|La rampe redevient lisse.
-enfant-m|On peut glisser !</t>
+narrateur|Ça file, tout d'un coup.</t>
         </is>
       </c>
       <c r="AX68" t="inlineStr">
@@ -13566,12 +13566,12 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>L'ombre violette touche déjà l'herbe. Le doudou dort dans le bac, tout sablé. Le doudou est. Aniss garde les mains, et attend. Il le veut, ce doudou ? Le doudou est tout sablé. On le tapote. Le sable tombe, un nuage minuscule. Nino le serre contre sa joue. Un lampadaire fait un petit tic. Il est prêt, maintenant. On grimpe, avec lui.</t>
+          <t>L'ombre violette touche déjà l'herbe. Le doudou dort dans le bac, tout sablé. Le doudou est. Aniss garde les mains, et attend. Il le veut, ce doudou ? Le doudou est tout sablé. On le tapote. Le sable tombe, un nuage minuscule. Nino le serre contre sa joue. Un lampadaire fait un petit tic. Il est prêt, maintenant. Ils glissent, le doudou entre eux.</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>L'ombre violette touche déjà l'herbe. Le doudou dort dans le bac, tout sablé. Le doudou est. Aniss garde les mains, et attend. Il le veut, ce doudou ? Le doudou est tout sablé. On le tapote. Le sable tombe, un nuage minuscule. Nino le serre contre sa joue. Un lampadaire fait un petit tic. Il est prêt, maintenant. On grimpe, avec lui.</t>
+          <t>L'ombre violette touche déjà l'herbe. Le doudou dort dans le bac, tout sablé. Le doudou est. Aniss garde les mains, et attend. Il le veut, ce doudou ? Le doudou est tout sablé. On le tapote. Le sable tombe, un nuage minuscule. Nino le serre contre sa joue. Un lampadaire fait un petit tic. Il est prêt, maintenant. Ils glissent, le doudou entre eux.</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -13717,7 +13717,7 @@
 narrateur|Nino le serre contre sa joue.
 narrateur|Un lampadaire fait un petit tic.
 maman|Il est prêt, maintenant.
-enfant-m|On grimpe, avec lui.</t>
+narrateur|Ils glissent, le doudou entre eux.</t>
         </is>
       </c>
       <c r="AX70" t="inlineStr">
@@ -14300,12 +14300,12 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Maintenant le toboggan refroidit. Le ballon rouge coince un barreau. Le ballon va. Aniss ouvre les mains, en bas, et attend. Tu le laisses dire ? Le ballon va tomber. Je suis là. Nino pousse, tout doux. Le rouge atterrit dans les mains d'Aniss. Un lampadaire fait un petit tic. Le chemin est libre. On monte, puis on glisse !</t>
+          <t>Maintenant le toboggan refroidit. Le ballon rouge coince un barreau. Le ballon va. Aniss ouvre les mains, en bas, et attend. Tu le laisses dire ? Le ballon va tomber. Je suis là. Nino pousse, tout doux. Le rouge atterrit dans les mains d'Aniss. Un lampadaire fait un petit tic. Le chemin est libre. Ils montent, puis ça dévale.</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>Maintenant le toboggan refroidit. Le ballon rouge coince un barreau. Le ballon va. Aniss ouvre les mains, en bas, et attend. Tu le laisses dire ? Le ballon va tomber. Je suis là. Nino pousse, tout doux. Le rouge atterrit dans les mains d'Aniss. Un lampadaire fait un petit tic. Le chemin est libre. On monte, puis on glisse !</t>
+          <t>Maintenant le toboggan refroidit. Le ballon rouge coince un barreau. Le ballon va. Aniss ouvre les mains, en bas, et attend. Tu le laisses dire ? Le ballon va tomber. Je suis là. Nino pousse, tout doux. Le rouge atterrit dans les mains d'Aniss. Un lampadaire fait un petit tic. Le chemin est libre. Ils montent, puis ça dévale.</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -14447,7 +14447,7 @@
 narrateur|Le rouge atterrit dans les mains d'Aniss.
 narrateur|Un lampadaire fait un petit tic.
 papa|Le chemin est libre.
-enfant-m|On monte, puis on glisse !</t>
+narrateur|Ils montent, puis ça dévale.</t>
         </is>
       </c>
       <c r="AX74" t="inlineStr">
@@ -14659,12 +14659,12 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>L'ombre violette touche déjà l'herbe. Le seau bleu pend près du haut. Le seau va. Aniss reste un barreau plus bas. On l'écoute, d'accord ? Le seau va nous aider. Je te le tends. Nino pousse le sable, tout lentement. Les grains tombent dans le bleu. Voilà le sable, déjà refroidi, tout fin. La rampe redevient glissante. À nous !</t>
+          <t>L'ombre violette touche déjà l'herbe. Le seau bleu pend près du haut. Le seau va. Aniss reste un barreau plus bas. On l'écoute, d'accord ? Le seau va nous aider. Je te le tends. Nino pousse le sable, tout lentement. Les grains tombent dans le bleu. Voilà le sable, déjà refroidi, tout fin. La rampe redevient glissante. Ils dévalent, le seau à la main.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>L'ombre violette touche déjà l'herbe. Le seau bleu pend près du haut. Le seau va. Aniss reste un barreau plus bas. On l'écoute, d'accord ? Le seau va nous aider. Je te le tends. Nino pousse le sable, tout lentement. Les grains tombent dans le bleu. Voilà le sable, déjà refroidi, tout fin. La rampe redevient glissante. À nous !</t>
+          <t>L'ombre violette touche déjà l'herbe. Le seau bleu pend près du haut. Le seau va. Aniss reste un barreau plus bas. On l'écoute, d'accord ? Le seau va nous aider. Je te le tends. Nino pousse le sable, tout lentement. Les grains tombent dans le bleu. Voilà le sable, déjà refroidi, tout fin. La rampe redevient glissante. Ils dévalent, le seau à la main.</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -14806,7 +14806,7 @@
 narrateur|Les grains tombent dans le bleu.
 narrateur|Voilà le sable, déjà refroidi, tout fin.
 maman|La rampe redevient glissante.
-enfant-m|À nous !</t>
+narrateur|Ils dévalent, le seau à la main.</t>
         </is>
       </c>
       <c r="AX76" t="inlineStr">
@@ -15018,12 +15018,12 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>La lumière devient orange, tout doux. Le doudou est coincé sur un barreau. Le doudou va. Aniss ne le prend pas, et attend. Sa phrase n'est pas finie. Le doudou va avec moi. Je te le passe. Nino le glisse sous son bras. Ils montent, barreau après barreau. Maintenant le toboggan refroidit. Vous y êtes, tout en haut. On glisse ensemble !</t>
+          <t>La lumière devient orange, tout doux. Le doudou est coincé sur un barreau. Le doudou va. Aniss ne le prend pas, et attend. Il cherche encore. Le doudou va avec moi. Je te le passe. Nino le glisse sous son bras. Ils montent, barreau après barreau. Maintenant le toboggan refroidit. Vous y êtes, tout en haut. Ils glissent, le doudou au milieu.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>La lumière devient orange, tout doux. Le doudou est coincé sur un barreau. Le doudou va. Aniss ne le prend pas, et attend. Sa phrase n'est pas finie. Le doudou va avec moi. Je te le passe. Nino le glisse sous son bras. Ils montent, barreau après barreau. Maintenant le toboggan refroidit. Vous y êtes, tout en haut. On glisse ensemble !</t>
+          <t>La lumière devient orange, tout doux. Le doudou est coincé sur un barreau. Le doudou va. Aniss ne le prend pas, et attend. Il cherche encore. Le doudou va avec moi. Je te le passe. Nino le glisse sous son bras. Ils montent, barreau après barreau. Maintenant le toboggan refroidit. Vous y êtes, tout en haut. Ils glissent, le doudou au milieu.</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -15158,14 +15158,14 @@
 narrateur|Le doudou est coincé sur un barreau.
 copain|Le doudou va.
 narrateur|Aniss ne le prend pas, et attend.
-maman|Sa phrase n'est pas finie.
+maman|Il cherche encore.
 copain|Le doudou va avec moi.
 enfant-m|Je te le passe.
 narrateur|Nino le glisse sous son bras.
 narrateur|Ils montent, barreau après barreau.
 narrateur|Maintenant le toboggan refroidit.
 papa|Vous y êtes, tout en haut.
-enfant-m|On glisse ensemble !</t>
+narrateur|Ils glissent, le doudou au milieu.</t>
         </is>
       </c>
       <c r="AX78" t="inlineStr">
@@ -16819,7 +16819,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -16869,6 +16869,13 @@
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>